<commit_message>
Update batch_27.xlsx and 03-ddl-data-types.pdf with new content
</commit_message>
<xml_diff>
--- a/batch_notes/batch_27.xlsx
+++ b/batch_notes/batch_27.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10617"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10625"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/ALI_2/work/acciojob/modules/sql/postgresql/batch_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E3AFCB-1852-F241-9373-EC3CC3748197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D5FFD1-C178-564C-84CD-919CB93B6A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="-2480" windowWidth="38400" windowHeight="21600" xr2:uid="{43D057EC-24A4-D14F-BD50-FDFE67984E9E}"/>
+    <workbookView xWindow="29400" yWindow="-2480" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{43D057EC-24A4-D14F-BD50-FDFE67984E9E}"/>
   </bookViews>
   <sheets>
     <sheet name="01" sheetId="1" r:id="rId1"/>
+    <sheet name="03" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
   <si>
     <t>RDBMS</t>
   </si>
@@ -69,6 +70,108 @@
   </si>
   <si>
     <t>Function</t>
+  </si>
+  <si>
+    <t>DDL</t>
+  </si>
+  <si>
+    <t>Data Types</t>
+  </si>
+  <si>
+    <t>Shiraj</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>Numeric</t>
+  </si>
+  <si>
+    <t>smallint</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>bigint</t>
+  </si>
+  <si>
+    <t>serial</t>
+  </si>
+  <si>
+    <t>bigserial</t>
+  </si>
+  <si>
+    <t>numeric</t>
+  </si>
+  <si>
+    <t>real</t>
+  </si>
+  <si>
+    <t>double_prec</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>char</t>
+  </si>
+  <si>
+    <t>varchar</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>2 GB</t>
+  </si>
+  <si>
+    <t>\0</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>5 Byte</t>
+  </si>
+  <si>
+    <t>7 Byte</t>
+  </si>
+  <si>
+    <t>Varing character</t>
+  </si>
+  <si>
+    <t>000111</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>TIME</t>
+  </si>
+  <si>
+    <t>TIMESTAMP</t>
+  </si>
+  <si>
+    <t>TIMESTAMPTZ</t>
+  </si>
+  <si>
+    <t>INTERVAL</t>
   </si>
 </sst>
 </file>
@@ -92,7 +195,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -100,12 +203,54 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1382,6 +1527,16 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B75C81F2-16C4-AA43-AAFC-971767DED54C}" name="Table1" displayName="Table1" ref="C6:C13" totalsRowShown="0">
+  <autoFilter ref="C6:C13" xr:uid="{B75C81F2-16C4-AA43-AAFC-971767DED54C}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{1BCB39CC-0060-EC4E-A86A-9DF4B948F471}" name="Column1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1759,4 +1914,197 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6423C9B5-2C8E-9C46-8123-8AB108F2818D}">
+  <dimension ref="B2:N25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="20.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C7">
+        <v>123</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="N11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="E12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M12">
+        <v>7</v>
+      </c>
+      <c r="N12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="E13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" t="s">
+        <v>29</v>
+      </c>
+      <c r="I13" t="s">
+        <v>30</v>
+      </c>
+      <c r="J13" t="s">
+        <v>31</v>
+      </c>
+      <c r="M13">
+        <v>7</v>
+      </c>
+      <c r="N13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="E18" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G18">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="C20" s="5">
+        <f ca="1">NOW()</f>
+        <v>46201.50655046296</v>
+      </c>
+    </row>
+    <row r="21" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="E21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="E22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="E23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="E24" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="E25" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>